<commit_message>
Deploying theChange or Fix made during production deployment
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aws-svc-rpa52d\Documents\UiPath\3043_LATAM_DataLoad\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DAE1DDB-10E7-40D6-9ED1-482F0783C24C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8179A41D-126D-4465-BABC-0B7CB2EE46FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="111">
   <si>
     <t>Name</t>
   </si>
@@ -156,7 +156,7 @@
   </si>
   <si>
     <t>Orchestrator queue Name. The value must match with the queue name defined on Orchestrator.</t>
-    <phoneticPr fontId="2"/>
+    <phoneticPr fontId="3"/>
   </si>
   <si>
     <t>excel</t>
@@ -235,9 +235,6 @@
   </si>
   <si>
     <t>3043_Mail_Account</t>
-  </si>
-  <si>
-    <t>3043_To_Exception_Mail_ID</t>
   </si>
   <si>
     <t>https://thermofisher.sharepoint.com/sites/FinanceCTDLatam/Shared%20Documents/Finance/Billing/{Year}/{Year}_{Month}/Revenue</t>
@@ -486,9 +483,6 @@
     <t>Successful_Email</t>
   </si>
   <si>
-    <t>nivedha.palani@thermofisher.com;nivedha.palani@thermofisher.com</t>
-  </si>
-  <si>
     <t>Email_Receipients</t>
   </si>
   <si>
@@ -647,16 +641,73 @@
   <si>
     <t>Mexico=Mexico,Mex,MEX,mexi;Argentina=Argentina,Arg,Arg1,Arg (2);Peru=Per,Peru;Colombia=Col,Colombia;Chile=Chi,Chile;Brazil=Bra,Brazil;Invoice Latam=Invoice Latam;Selectable Table =Selectable Table</t>
   </si>
+  <si>
+    <t>Email_ExceptionPrevalid</t>
+  </si>
+  <si>
+    <t>&lt;html&gt;
+&lt;body style="font-family: Arial, sans-serif; font-size:14px; color:#333;"&gt;
+&lt;div style="background-color:#C00000; color:white; padding:10px; font-size:17px; font-weight:bold;"&gt;
+    LATAM Data Validation - Prevalidation Failed
+&lt;/div&gt;
+&lt;br&gt;
+&lt;p&gt;Hi Team,&lt;/p&gt;
+&lt;p&gt;
+The LATAM Revenue and Invoice validation process could not be initiated for &lt;b&gt;{{MONTH}}&lt;/b&gt;
+because an error occurred during the prevalidation / initialization stage.
+&lt;/p&gt;
+&lt;p&gt;
+The process has been stopped due to the above error. Please review the details and take the necessary corrective action before restarting the process.
+&lt;/p&gt;
+&lt;table style="border-collapse:collapse; width:100%;"&gt;
+&lt;tr style="background-color:#F4CCCC;"&gt;
+    &lt;th style="border:1px solid #E6B8B7; padding:8px; text-align:left;"&gt;Process&lt;/th&gt;
+    &lt;th style="border:1px solid #E6B8B7; padding:8px; text-align:left;"&gt;Status&lt;/th&gt;
+    &lt;th style="border:1px solid #E6B8B7; padding:8px; text-align:left;"&gt;Error Details&lt;/th&gt;
+&lt;/tr&gt;
+&lt;tr&gt;
+    &lt;td style="border:1px solid #E6B8B7; padding:8px;"&gt;
+        Revenue &amp; Invoice Validation
+    &lt;/td&gt;
+    &lt;td style="border:1px solid #E6B8B7; padding:8px; font-weight:bold; color:#C00000;"&gt;
+        Prevalidation Failed
+    &lt;/td&gt;
+    &lt;td style="border:1px solid #E6B8B7; padding:8px;"&gt;
+        {{EXCEPTION_MESSAGE}}
+    &lt;/td&gt;
+&lt;/tr&gt;
+&lt;/table&gt;
+&lt;br&gt;
+&lt;p&gt;
+Regards,&lt;br&gt;
+Automation Team
+&lt;/p&gt;
+&lt;/body&gt;
+&lt;/html&gt;</t>
+  </si>
+  <si>
+    <t>RetryInterval</t>
+  </si>
+  <si>
+    <t>Diana.Austria@thermofisher.com;pedro.nogueira@thermofisher.com;norberto.camposdiaz@thermofisher.com;suraj.jain@thermofisher.com;sagar.kurhekar@thermofisher.com;nivedha.palani@thermofisher.com</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -707,6 +758,14 @@
       <color theme="10"/>
       <name val="Calibri"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -716,7 +775,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -724,33 +783,65 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="3" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="11">
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
+    <cellStyle name="Hyperlink 2" xfId="5" xr:uid="{22FEAACD-2E5D-4E97-8E0C-A12DE51800CA}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{9F090F5F-5753-47D9-8210-768656CA164E}"/>
+    <cellStyle name="Normal 2 2" xfId="9" xr:uid="{27BA1CE1-0C19-49B8-92D4-53353E07F8BB}"/>
+    <cellStyle name="Normal 2 3" xfId="7" xr:uid="{827354D1-14E8-4326-B25E-51F4517FCF7A}"/>
     <cellStyle name="Normal 3" xfId="1" xr:uid="{A98D3C50-28F7-4950-A674-469B8B9C40F3}"/>
+    <cellStyle name="Normal 4" xfId="6" xr:uid="{7CFD1B52-7B92-46E8-86A8-0F979F3F5DDD}"/>
+    <cellStyle name="Normal 5" xfId="8" xr:uid="{4EFC079D-ED92-4573-BF08-33792BED23EC}"/>
+    <cellStyle name="Normal 6" xfId="10" xr:uid="{FF5E97E1-4478-43F7-BFCB-3AF88EE9D4AD}"/>
+    <cellStyle name="Normal 7" xfId="4" xr:uid="{88BA6689-3B89-4FCC-BF4B-81E47217FB66}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1177,7 +1268,7 @@
         <v>55</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>40</v>
@@ -1185,19 +1276,26 @@
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" t="s">
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B10" s="12">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26" s="10" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A11" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>105</v>
+      <c r="B11" s="11" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1">
@@ -1213,31 +1311,31 @@
         <v>50</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>94</v>
-      </c>
-      <c r="B14" t="s">
-        <v>93</v>
+        <v>92</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B15" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B16" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
@@ -1250,59 +1348,66 @@
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" t="s">
+        <v>86</v>
+      </c>
+      <c r="B18" s="8" t="s">
         <v>87</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="14.25" customHeight="1"/>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A22" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>108</v>
+      </c>
+    </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
       <c r="A23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" t="s">
         <v>81</v>
-      </c>
-      <c r="B23" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" t="s">
+        <v>82</v>
+      </c>
+      <c r="B24" s="7" t="s">
         <v>83</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
@@ -1310,7 +1415,7 @@
         <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.25" customHeight="1">
@@ -1318,7 +1423,7 @@
         <v>59</v>
       </c>
       <c r="B27" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
@@ -1326,7 +1431,7 @@
         <v>60</v>
       </c>
       <c r="B28" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
@@ -1334,7 +1439,7 @@
         <v>61</v>
       </c>
       <c r="B29" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
@@ -1342,47 +1447,47 @@
         <v>62</v>
       </c>
       <c r="B30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B31" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
+        <v>74</v>
+      </c>
+      <c r="B34" t="s">
         <v>75</v>
-      </c>
-      <c r="B34" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="14.25" customHeight="1"/>
@@ -2297,7 +2402,7 @@
     <row r="945" ht="14.25" customHeight="1"/>
     <row r="946" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="2"/>
+  <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3409,7 +3514,7 @@
     <row r="972" ht="14.25" customHeight="1"/>
     <row r="973" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="2"/>
+  <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3418,7 +3523,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr codeName="Sheet3"/>
-  <dimension ref="A1:Z983"/>
+  <dimension ref="A1:Z982"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="31.85546875" customWidth="1"/>
@@ -3430,7 +3535,7 @@
   <sheetData>
     <row r="1" spans="1:26" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -3466,10 +3571,10 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C2" s="2"/>
     </row>
@@ -3510,18 +3615,10 @@
       <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A7" t="s">
-        <v>67</v>
-      </c>
-      <c r="B7" t="s">
-        <v>67</v>
-      </c>
-      <c r="C7" s="2"/>
-    </row>
-    <row r="8" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="2"/>
-    </row>
+      <c r="A7" s="3"/>
+      <c r="B7" s="2"/>
+    </row>
+    <row r="8" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="9" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="10" spans="1:26" ht="14.25" customHeight="1"/>
     <row r="11" spans="1:26" ht="14.25" customHeight="1"/>
@@ -4496,9 +4593,8 @@
     <row r="980" ht="14.25" customHeight="1"/>
     <row r="981" ht="14.25" customHeight="1"/>
     <row r="982" ht="14.25" customHeight="1"/>
-    <row r="983" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="2"/>
+  <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Changes Made to set the default run month.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aws-svc-rpa52d\Documents\UiPath\3043_LATAM_DataLoad\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8179A41D-126D-4465-BABC-0B7CB2EE46FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C16012-07D2-40AF-A7CD-4B0F2976310F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="113">
   <si>
     <t>Name</t>
   </si>
@@ -690,6 +690,12 @@
   </si>
   <si>
     <t>Diana.Austria@thermofisher.com;pedro.nogueira@thermofisher.com;norberto.camposdiaz@thermofisher.com;suraj.jain@thermofisher.com;sagar.kurhekar@thermofisher.com;nivedha.palani@thermofisher.com</t>
+  </si>
+  <si>
+    <t>AWSU1-0JWUIA16P</t>
+  </si>
+  <si>
+    <t>OrchestratorQueueFolderDev</t>
   </si>
 </sst>
 </file>
@@ -1154,7 +1160,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Z946"/>
+  <dimension ref="A1:Z947"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="35.28515625" customWidth="1"/>
@@ -1279,218 +1285,225 @@
         <v>88</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A10" t="s">
+        <v>112</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" s="3" t="s">
+    <row r="11" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A11" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B11" s="12">
         <v>5</v>
       </c>
     </row>
-    <row r="11" spans="1:26" s="10" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A11" s="10" t="s">
+    <row r="12" spans="1:26" s="10" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A12" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B12" s="11" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="12" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>104</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>92</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>110</v>
+        <v>50</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>100</v>
-      </c>
-      <c r="B15" t="s">
-        <v>101</v>
+        <v>92</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
       <c r="A16" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B16" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s">
-        <v>53</v>
+        <v>102</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" t="s">
+        <v>54</v>
+      </c>
+      <c r="B18" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A19" t="s">
         <v>86</v>
       </c>
-      <c r="B18" s="8" t="s">
+      <c r="B19" s="8" t="s">
         <v>87</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A19" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="B19" s="8" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A23" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="B22" s="9" t="s">
+      <c r="B23" s="9" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A23" t="s">
-        <v>80</v>
-      </c>
-      <c r="B23" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>82</v>
-      </c>
-      <c r="B24" s="7" t="s">
-        <v>83</v>
+        <v>80</v>
+      </c>
+      <c r="B24" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>85</v>
-      </c>
-      <c r="B25" t="s">
-        <v>84</v>
+        <v>82</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>85</v>
       </c>
       <c r="B26" t="s">
-        <v>67</v>
+        <v>84</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B27" t="s">
-        <v>105</v>
+        <v>67</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B29" t="s">
-        <v>78</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B30" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>97</v>
+        <v>62</v>
       </c>
       <c r="B31" t="s">
-        <v>98</v>
+        <v>79</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>68</v>
+        <v>97</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>98</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B33" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B34" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
+        <v>74</v>
+      </c>
+      <c r="B35" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="14.25" customHeight="1">
+      <c r="A36" t="s">
         <v>77</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B36" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="37" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="38" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="39" spans="1:2" ht="14.25" customHeight="1"/>
@@ -2401,6 +2414,7 @@
     <row r="944" ht="14.25" customHeight="1"/>
     <row r="945" ht="14.25" customHeight="1"/>
     <row r="946" ht="14.25" customHeight="1"/>
+    <row r="947" ht="14.25" customHeight="1"/>
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Comit after adding missing dependency.
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aws-svc-rpa52d\Documents\UiPath\3043_LATAM_DataLoad\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42C16012-07D2-40AF-A7CD-4B0F2976310F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{995FBC67-7605-499C-9BE3-CFB3C785080D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="111">
   <si>
     <t>Name</t>
   </si>
@@ -156,7 +156,7 @@
   </si>
   <si>
     <t>Orchestrator queue Name. The value must match with the queue name defined on Orchestrator.</t>
-    <phoneticPr fontId="3"/>
+    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>excel</t>
@@ -483,6 +483,9 @@
     <t>Successful_Email</t>
   </si>
   <si>
+    <t>nivedha.palani@thermofisher.com;nivedha.palani@thermofisher.com</t>
+  </si>
+  <si>
     <t>Email_Receipients</t>
   </si>
   <si>
@@ -633,9 +636,6 @@
     <t xml:space="preserve">3043 LATAM Data Load |Business Exception </t>
   </si>
   <si>
-    <t xml:space="preserve">3043  LATAM Data Load |System Exception </t>
-  </si>
-  <si>
     <t>Mexico=Mexico,Mex,MEX,mexi;Arg1=Arg,Arg1,Arg (2);Per=Per,Peru;Col=Col,Colombia;Chi=Chi,Chile;Bra=Bra,Brazil;Bra TP=Bra TP;HFM (Datos)=HFM (Datos),HFM;Selectable Table =Selectable Table</t>
   </si>
   <si>
@@ -689,31 +689,18 @@
     <t>RetryInterval</t>
   </si>
   <si>
-    <t>Diana.Austria@thermofisher.com;pedro.nogueira@thermofisher.com;norberto.camposdiaz@thermofisher.com;suraj.jain@thermofisher.com;sagar.kurhekar@thermofisher.com;nivedha.palani@thermofisher.com</t>
-  </si>
-  <si>
-    <t>AWSU1-0JWUIA16P</t>
-  </si>
-  <si>
-    <t>OrchestratorQueueFolderDev</t>
+    <t>3043  LATAM Data Load |Business Exception</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -764,14 +751,6 @@
       <color theme="10"/>
       <name val="Calibri"/>
     </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -799,55 +778,38 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="11">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="3" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="3" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="4" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="11">
+  <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="3" builtinId="8"/>
-    <cellStyle name="Hyperlink 2" xfId="5" xr:uid="{22FEAACD-2E5D-4E97-8E0C-A12DE51800CA}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{9F090F5F-5753-47D9-8210-768656CA164E}"/>
-    <cellStyle name="Normal 2 2" xfId="9" xr:uid="{27BA1CE1-0C19-49B8-92D4-53353E07F8BB}"/>
-    <cellStyle name="Normal 2 3" xfId="7" xr:uid="{827354D1-14E8-4326-B25E-51F4517FCF7A}"/>
     <cellStyle name="Normal 3" xfId="1" xr:uid="{A98D3C50-28F7-4950-A674-469B8B9C40F3}"/>
-    <cellStyle name="Normal 4" xfId="6" xr:uid="{7CFD1B52-7B92-46E8-86A8-0F979F3F5DDD}"/>
-    <cellStyle name="Normal 5" xfId="8" xr:uid="{4EFC079D-ED92-4573-BF08-33792BED23EC}"/>
-    <cellStyle name="Normal 6" xfId="10" xr:uid="{FF5E97E1-4478-43F7-BFCB-3AF88EE9D4AD}"/>
-    <cellStyle name="Normal 7" xfId="4" xr:uid="{88BA6689-3B89-4FCC-BF4B-81E47217FB66}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1160,7 +1122,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:Z947"/>
+  <dimension ref="A1:Z946"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="35.28515625" customWidth="1"/>
@@ -1285,55 +1247,55 @@
         <v>88</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>111</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>112</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="11" spans="1:26" ht="14.25" customHeight="1">
-      <c r="A11" s="3" t="s">
+      <c r="A10" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B10" s="12">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="1:26" s="10" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A12" s="10" t="s">
+    <row r="11" spans="1:26" s="10" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A11" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>103</v>
+      <c r="B11" s="11" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" ht="14.25" customHeight="1">
+      <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>49</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1">
       <c r="A14" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>104</v>
+        <v>93</v>
+      </c>
+      <c r="B14" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1">
       <c r="A15" t="s">
-        <v>92</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>110</v>
+        <v>101</v>
+      </c>
+      <c r="B15" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1">
@@ -1341,169 +1303,162 @@
         <v>100</v>
       </c>
       <c r="B16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="14.25" customHeight="1">
       <c r="A17" t="s">
-        <v>99</v>
+        <v>54</v>
       </c>
       <c r="B17" t="s">
-        <v>102</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="14.25" customHeight="1">
       <c r="A18" t="s">
-        <v>54</v>
-      </c>
-      <c r="B18" t="s">
-        <v>53</v>
+        <v>86</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A19" t="s">
-        <v>86</v>
+      <c r="A19" s="2" t="s">
+        <v>90</v>
       </c>
       <c r="B19" s="8" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="14.25" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="14.25" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="14.25" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>96</v>
+        <v>107</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A23" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>108</v>
+      <c r="A23" t="s">
+        <v>80</v>
+      </c>
+      <c r="B23" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="14.25" customHeight="1">
       <c r="A24" t="s">
-        <v>80</v>
-      </c>
-      <c r="B24" t="s">
-        <v>81</v>
+        <v>82</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="14.25" customHeight="1">
       <c r="A25" t="s">
-        <v>82</v>
-      </c>
-      <c r="B25" s="7" t="s">
-        <v>83</v>
+        <v>85</v>
+      </c>
+      <c r="B25" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="14.25" customHeight="1">
       <c r="A26" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="B26" t="s">
-        <v>84</v>
+        <v>67</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="14.25" customHeight="1">
       <c r="A27" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B27" t="s">
-        <v>67</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="14.25" customHeight="1">
       <c r="A28" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B28" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="14.25" customHeight="1">
       <c r="A29" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B29" t="s">
-        <v>106</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="14.25" customHeight="1">
       <c r="A30" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="14.25" customHeight="1">
       <c r="A31" t="s">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="B31" t="s">
-        <v>79</v>
+        <v>99</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="14.25" customHeight="1">
       <c r="A32" t="s">
-        <v>97</v>
+        <v>68</v>
       </c>
       <c r="B32" t="s">
-        <v>98</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="14.25" customHeight="1">
       <c r="A33" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B34" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="14.25" customHeight="1">
       <c r="A35" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="14.25" customHeight="1">
-      <c r="A36" t="s">
-        <v>77</v>
-      </c>
-      <c r="B36" t="s">
         <v>76</v>
       </c>
     </row>
+    <row r="36" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="37" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="38" spans="1:2" ht="14.25" customHeight="1"/>
     <row r="39" spans="1:2" ht="14.25" customHeight="1"/>
@@ -2414,9 +2369,8 @@
     <row r="944" ht="14.25" customHeight="1"/>
     <row r="945" ht="14.25" customHeight="1"/>
     <row r="946" ht="14.25" customHeight="1"/>
-    <row r="947" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3528,7 +3482,7 @@
     <row r="972" ht="14.25" customHeight="1"/>
     <row r="973" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -4608,7 +4562,7 @@
     <row r="981" ht="14.25" customHeight="1"/>
     <row r="982" ht="14.25" customHeight="1"/>
   </sheetData>
-  <phoneticPr fontId="3"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>